<commit_message>
Phase one major excel QC on the way
</commit_message>
<xml_diff>
--- a/input/12_Loadshapes.xlsx
+++ b/input/12_Loadshapes.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29421"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="104" documentId="11_CBBF0E96895A3475DC461CCF33652BCD3DED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A6BBD62-4507-402A-A713-F918B999D1E2}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/market_inputs/input/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="113" documentId="11_CBBF0E96895A3475DC461CCF33652BCD3DED4083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A750A81B-905E-4958-A9E1-1155B6E43FC1}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loadshapes" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -77,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="44">
   <si>
     <t>condition_name</t>
   </si>
@@ -197,20 +203,28 @@
   </si>
   <si>
     <t>Wall Insulation_Res, E - Cool [Elec Heating] _Multifamily_Cooling</t>
+  </si>
+  <si>
+    <t>Load shapes are only needed for the efficient technology</t>
+  </si>
+  <si>
+    <t>Will need to add the list of efficient measures and this sheet's output to the module Matt requested</t>
+  </si>
+  <si>
+    <t>insulation_natural_gas_efficient_residential</t>
+  </si>
+  <si>
+    <t>HERS_electric_efficient_residential</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0000_);[Red]\(#,##0.0000\)"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -257,7 +271,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,12 +281,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="43"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -314,13 +322,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -332,23 +339,11 @@
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Comma" xfId="3" builtinId="3"/>
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal_PST Maine Triennial Plan" xfId="2" xr:uid="{14ECC767-CF4D-4D2F-A4A8-0F2E3142C260}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
@@ -683,8 +678,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.140625" customWidth="1"/>
@@ -697,7 +692,7 @@
     <col min="11" max="11" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -738,7 +733,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
@@ -748,38 +743,39 @@
       <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="3">
         <v>7.8778425231575966E-3</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="3">
         <v>1.8345799297094345E-2</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="3">
         <v>0.28181183338165283</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="3">
         <v>0.36880850791931152</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="3">
         <v>0.12986405193805695</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I2" s="3">
         <v>0.19329194724559784</v>
       </c>
-      <c r="J2" s="9">
+      <c r="J2" s="3">
         <v>0</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="3">
         <v>0.3810066126706862</v>
       </c>
-      <c r="L2" s="9">
+      <c r="L2" s="3">
         <v>0</v>
       </c>
-      <c r="M2" s="9">
+      <c r="M2" s="3">
         <v>0.3810066126706862</v>
       </c>
-    </row>
-    <row r="3" spans="1:13">
+      <c r="N2" s="3"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>16</v>
       </c>
@@ -789,38 +785,39 @@
       <c r="C3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="3">
         <v>7.8778425231575966E-3</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="3">
         <v>1.8345799297094345E-2</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="3">
         <v>0.28181183338165283</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="3">
         <v>0.36880850791931152</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="3">
         <v>0.12986405193805695</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="3">
         <v>0.19329194724559784</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="3">
         <v>0</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="3">
         <v>0.3810066126706862</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L3" s="3">
         <v>0</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="3">
         <v>0.3810066126706862</v>
       </c>
-    </row>
-    <row r="4" spans="1:13">
+      <c r="N3" s="3"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>18</v>
       </c>
@@ -830,38 +827,39 @@
       <c r="C4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="3">
         <v>7.8778425231575966E-3</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="3">
         <v>1.8345799297094345E-2</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="3">
         <v>0.28181183338165283</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="3">
         <v>0.36880850791931152</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="3">
         <v>0.12986405193805695</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="3">
         <v>0.19329194724559784</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="3">
         <v>0</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="3">
         <v>0.3810066126706862</v>
       </c>
-      <c r="L4" s="9">
+      <c r="L4" s="3">
         <v>0</v>
       </c>
-      <c r="M4" s="9">
+      <c r="M4" s="3">
         <v>0.3810066126706862</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="N4" s="3"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>19</v>
       </c>
@@ -871,38 +869,39 @@
       <c r="C5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="3">
         <v>0.49062061309814453</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="3">
         <v>0.37157672643661499</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="3">
         <v>2.0993791520595551E-2</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="3">
         <v>2.6758521795272827E-2</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="3">
         <v>4.8400141298770905E-2</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="3">
         <v>4.1650202125310898E-2</v>
       </c>
-      <c r="J5" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K5">
+      <c r="J5" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K5" s="3">
         <v>0</v>
       </c>
-      <c r="L5" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M5">
+      <c r="L5" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M5" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13">
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>21</v>
       </c>
@@ -912,38 +911,39 @@
       <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="3">
         <v>0.49062061309814453</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="3">
         <v>0.37157672643661499</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="3">
         <v>2.0993791520595551E-2</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="3">
         <v>2.6758521795272827E-2</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="3">
         <v>4.8400141298770905E-2</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="3">
         <v>4.1650202125310898E-2</v>
       </c>
-      <c r="J6" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K6">
+      <c r="J6" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K6" s="3">
         <v>0</v>
       </c>
-      <c r="L6" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M6">
+      <c r="L6" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M6" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:13">
+      <c r="N6" s="3"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -953,38 +953,39 @@
       <c r="C7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="3">
         <v>0.49062061309814453</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="3">
         <v>0.37157672643661499</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="3">
         <v>2.0993791520595551E-2</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="3">
         <v>2.6758521795272827E-2</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="3">
         <v>4.8400141298770905E-2</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="3">
         <v>4.1650202125310898E-2</v>
       </c>
-      <c r="J7" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K7">
+      <c r="J7" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K7" s="3">
         <v>0</v>
       </c>
-      <c r="L7" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M7">
+      <c r="L7" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M7" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:13">
+      <c r="N7" s="3"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>24</v>
       </c>
@@ -994,38 +995,39 @@
       <c r="C8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="3">
         <v>0.49062061309814453</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <v>0.37157672643661499</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="3">
         <v>2.0993791520595551E-2</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="3">
         <v>2.6758521795272827E-2</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="3">
         <v>4.8400141298770905E-2</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="3">
         <v>4.1650202125310898E-2</v>
       </c>
-      <c r="J8" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K8">
+      <c r="J8" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K8" s="3">
         <v>0</v>
       </c>
-      <c r="L8" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M8">
+      <c r="L8" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M8" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:13">
+      <c r="N8" s="3"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>25</v>
       </c>
@@ -1035,38 +1037,39 @@
       <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <v>0.49062061309814453</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="3">
         <v>0.37157672643661499</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="3">
         <v>2.0993791520595551E-2</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="3">
         <v>2.6758521795272827E-2</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="3">
         <v>4.8400141298770905E-2</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="3">
         <v>4.1650202125310898E-2</v>
       </c>
-      <c r="J9" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K9">
+      <c r="J9" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K9" s="3">
         <v>0</v>
       </c>
-      <c r="L9" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M9">
+      <c r="L9" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M9" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>27</v>
       </c>
@@ -1076,38 +1079,39 @@
       <c r="C10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <v>0.2208627313375473</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="3">
         <v>0.23739945888519287</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="3">
         <v>9.5015056431293488E-2</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="3">
         <v>0.11033865064382553</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="3">
         <v>0.16472350060939789</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="3">
         <v>0.17166060209274292</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="3">
         <v>1.186104</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="3">
         <v>0.88826399999999994</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="3">
         <v>1.186104</v>
       </c>
-      <c r="M10" s="8">
+      <c r="M10" s="3">
         <v>0.88826399999999994</v>
       </c>
-    </row>
-    <row r="11" spans="1:13">
+      <c r="N10" s="3"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>30</v>
       </c>
@@ -1117,38 +1121,39 @@
       <c r="C11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="3">
         <v>0.2208627313375473</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="3">
         <v>0.23739945888519287</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="3">
         <v>9.5015056431293488E-2</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="3">
         <v>0.11033865064382553</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="3">
         <v>0.16472350060939789</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="3">
         <v>0.17166060209274292</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="3">
         <v>1.186104</v>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="3">
         <v>0.88826399999999994</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L11" s="3">
         <v>1.186104</v>
       </c>
-      <c r="M11" s="8">
+      <c r="M11" s="3">
         <v>0.88826399999999994</v>
       </c>
-    </row>
-    <row r="12" spans="1:13">
+      <c r="N11" s="3"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>31</v>
       </c>
@@ -1158,38 +1163,39 @@
       <c r="C12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="3">
         <v>0.2208627313375473</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="3">
         <v>0.23739945888519287</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="3">
         <v>9.5015056431293488E-2</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="3">
         <v>0.11033865064382553</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="3">
         <v>0.16472350060939789</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I12" s="3">
         <v>0.17166060209274292</v>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="3">
         <v>1.186104</v>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="3">
         <v>0.88826399999999994</v>
       </c>
-      <c r="L12" s="10">
+      <c r="L12" s="3">
         <v>1.186104</v>
       </c>
-      <c r="M12" s="8">
+      <c r="M12" s="3">
         <v>0.88826399999999994</v>
       </c>
-    </row>
-    <row r="13" spans="1:13">
+      <c r="N12" s="3"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>32</v>
       </c>
@@ -1199,85 +1205,87 @@
       <c r="C13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="3">
         <v>0.2208627313375473</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="3">
         <v>0.23739945888519287</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="3">
         <v>9.5015056431293488E-2</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="3">
         <v>0.11033865064382553</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="3">
         <v>0.16472350060939789</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="3">
         <v>0.17166060209274292</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="3">
         <v>1.186104</v>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="3">
         <v>0.88826399999999994</v>
       </c>
-      <c r="L13" s="10">
+      <c r="L13" s="3">
         <v>1.186104</v>
       </c>
-      <c r="M13" s="8">
+      <c r="M13" s="3">
         <v>0.88826399999999994</v>
       </c>
-    </row>
-    <row r="14" spans="1:13">
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="3">
         <f>AVERAGE(Sheet2!B1:B2)</f>
         <v>0.24213783419691026</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="3">
         <f>AVERAGE(Sheet2!C1:C2)</f>
         <v>0.19750067032873631</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="3">
         <f>AVERAGE(Sheet2!D1:D2)</f>
         <v>0.15198543108999729</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <f>AVERAGE(Sheet2!E1:E2)</f>
         <v>0.20428621582686901</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="3">
         <f>AVERAGE(Sheet2!F1:F2)</f>
         <v>8.8423352688550949E-2</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="3">
         <f>AVERAGE(Sheet2!G1:G2)</f>
         <v>0.11566651985049248</v>
       </c>
-      <c r="J14" s="9">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K14" s="9">
+      <c r="J14" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K14" s="3">
         <v>0.3810066126706862</v>
       </c>
-      <c r="L14" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M14" s="8">
+      <c r="L14" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M14" s="3">
         <v>0.3810066126706862</v>
       </c>
-    </row>
-    <row r="15" spans="1:13">
+      <c r="N14" s="3"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>36</v>
       </c>
@@ -1287,38 +1295,39 @@
       <c r="C15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="3">
         <v>0.24213783419691026</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="3">
         <v>0.19750067032873631</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="3">
         <v>0.15198543108999729</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="3">
         <v>0.20428621582686901</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="3">
         <v>8.8423352688550949E-2</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="3">
         <v>0.11566651985049248</v>
       </c>
-      <c r="J15" s="9">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K15" s="9">
+      <c r="J15" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K15" s="3">
         <v>0.3810066126706862</v>
       </c>
-      <c r="L15" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M15" s="8">
+      <c r="L15" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M15" s="3">
         <v>0.3810066126706862</v>
       </c>
-    </row>
-    <row r="16" spans="1:13">
+      <c r="N15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>37</v>
       </c>
@@ -1328,245 +1337,189 @@
       <c r="C16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="3">
         <v>0.24213783419691026</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="3">
         <v>0.19750067032873631</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3">
         <v>0.15198543108999729</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>0.20428621582686901</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="3">
         <v>8.8423352688550949E-2</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="3">
         <v>0.11566651985049248</v>
       </c>
-      <c r="J16" s="9">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="K16" s="9">
+      <c r="J16" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K16" s="3">
         <v>0.3810066126706862</v>
       </c>
-      <c r="L16" s="10">
-        <v>0.37286116117435042</v>
-      </c>
-      <c r="M16" s="8">
+      <c r="L16" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M16" s="3">
         <v>0.3810066126706862</v>
       </c>
-    </row>
-    <row r="20" spans="4:11">
-      <c r="D20" s="11">
-        <v>0.06</v>
-      </c>
-      <c r="E20" s="11">
-        <v>0.04</v>
-      </c>
-      <c r="F20" s="11">
-        <v>0.06</v>
-      </c>
-      <c r="G20" s="11">
-        <v>0.04</v>
-      </c>
-      <c r="H20" s="11">
-        <v>0.04</v>
-      </c>
-      <c r="I20" s="11">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="21" spans="4:11">
-      <c r="D21">
-        <f>SUMPRODUCT(D2:I2,D$20:I$20)</f>
-        <v>4.5793792810291056E-2</v>
-      </c>
-      <c r="E21">
-        <f>D21*100</f>
-        <v>4.5793792810291052</v>
-      </c>
-      <c r="F21">
-        <f>E21*(1-G$21)</f>
-        <v>4.1475438148280599</v>
-      </c>
-      <c r="G21" s="12">
-        <v>9.430000000000005E-2</v>
-      </c>
-      <c r="J21">
-        <v>89.69</v>
-      </c>
-      <c r="K21">
-        <v>9.430000000000005E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="4:11">
-      <c r="D22">
-        <f t="shared" ref="D22:D32" si="0">SUMPRODUCT(D3:I3,D$20:I$20)</f>
-        <v>4.5793792810291056E-2</v>
-      </c>
-      <c r="E22">
-        <f t="shared" ref="E22:E32" si="1">D22*100</f>
-        <v>4.5793792810291052</v>
-      </c>
-      <c r="F22">
-        <f t="shared" ref="F22:F32" si="2">E22*(1-G$21)</f>
-        <v>4.1475438148280599</v>
-      </c>
-      <c r="J22">
-        <f>J21*J5*(1-K21)</f>
-        <v>30.288344721165387</v>
-      </c>
-    </row>
-    <row r="23" spans="4:11">
-      <c r="D23">
-        <f t="shared" si="0"/>
-        <v>4.5793792810291056E-2</v>
-      </c>
-      <c r="E23">
-        <f t="shared" si="1"/>
-        <v>4.5793792810291052</v>
-      </c>
-      <c r="F23">
-        <f t="shared" si="2"/>
-        <v>4.1475438148280599</v>
-      </c>
-      <c r="J23">
-        <f>J22*75</f>
-        <v>2271.6258540874042</v>
-      </c>
-    </row>
-    <row r="24" spans="4:11">
-      <c r="D24">
-        <f t="shared" si="0"/>
-        <v>5.0232287943363194E-2</v>
-      </c>
-      <c r="E24">
-        <f t="shared" si="1"/>
-        <v>5.023228794336319</v>
-      </c>
-      <c r="F24">
-        <f t="shared" si="2"/>
-        <v>4.549538319030404</v>
-      </c>
-    </row>
-    <row r="25" spans="4:11">
-      <c r="D25">
-        <f t="shared" si="0"/>
-        <v>5.0232287943363194E-2</v>
-      </c>
-      <c r="E25">
-        <f t="shared" si="1"/>
-        <v>5.023228794336319</v>
-      </c>
-      <c r="F25">
-        <f t="shared" si="2"/>
-        <v>4.549538319030404</v>
-      </c>
-    </row>
-    <row r="26" spans="4:11">
-      <c r="D26">
-        <f t="shared" si="0"/>
-        <v>5.0232287943363194E-2</v>
-      </c>
-      <c r="E26">
-        <f t="shared" si="1"/>
-        <v>5.023228794336319</v>
-      </c>
-      <c r="F26">
-        <f t="shared" si="2"/>
-        <v>4.549538319030404</v>
-      </c>
-    </row>
-    <row r="27" spans="4:11">
-      <c r="D27">
-        <f t="shared" si="0"/>
-        <v>5.0232287943363194E-2</v>
-      </c>
-      <c r="E27">
-        <f t="shared" si="1"/>
-        <v>5.023228794336319</v>
-      </c>
-      <c r="F27">
-        <f t="shared" si="2"/>
-        <v>4.549538319030404</v>
-      </c>
-    </row>
-    <row r="28" spans="4:11">
-      <c r="D28">
-        <f t="shared" si="0"/>
-        <v>5.0232287943363194E-2</v>
-      </c>
-      <c r="E28">
-        <f t="shared" si="1"/>
-        <v>5.023228794336319</v>
-      </c>
-      <c r="F28">
-        <f t="shared" si="2"/>
-        <v>4.549538319030404</v>
-      </c>
-    </row>
-    <row r="29" spans="4:11">
-      <c r="D29">
-        <f t="shared" si="0"/>
-        <v>4.6317555755376813E-2</v>
-      </c>
-      <c r="E29">
-        <f t="shared" si="1"/>
-        <v>4.6317555755376816</v>
-      </c>
-      <c r="F29">
-        <f t="shared" si="2"/>
-        <v>4.1949810247644779</v>
-      </c>
-    </row>
-    <row r="30" spans="4:11">
-      <c r="D30">
-        <f t="shared" si="0"/>
-        <v>4.6317555755376813E-2</v>
-      </c>
-      <c r="E30">
-        <f t="shared" si="1"/>
-        <v>4.6317555755376816</v>
-      </c>
-      <c r="F30">
-        <f t="shared" si="2"/>
-        <v>4.1949810247644779</v>
-      </c>
-    </row>
-    <row r="31" spans="4:11">
-      <c r="D31">
-        <f t="shared" si="0"/>
-        <v>4.6317555755376813E-2</v>
-      </c>
-      <c r="E31">
-        <f t="shared" si="1"/>
-        <v>4.6317555755376816</v>
-      </c>
-      <c r="F31">
-        <f t="shared" si="2"/>
-        <v>4.1949810247644779</v>
-      </c>
-    </row>
-    <row r="32" spans="4:11">
-      <c r="D32">
-        <f t="shared" si="0"/>
-        <v>4.6317555755376813E-2</v>
-      </c>
-      <c r="E32">
-        <f t="shared" si="1"/>
-        <v>4.6317555755376816</v>
-      </c>
-      <c r="F32">
-        <f t="shared" si="2"/>
-        <v>4.1949810247644779</v>
-      </c>
+      <c r="N16" s="3"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.24213783419691026</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.19750067032873631</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0.15198543108999729</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0.20428621582686901</v>
+      </c>
+      <c r="H17" s="3">
+        <v>8.8423352688550949E-2</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0.11566651985049248</v>
+      </c>
+      <c r="J17" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0.3810066126706862</v>
+      </c>
+      <c r="L17" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M17" s="3">
+        <v>0.3810066126706862</v>
+      </c>
+      <c r="N17" s="3"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.24213783419691026</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0.19750067032873631</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0.15198543108999729</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0.20428621582686901</v>
+      </c>
+      <c r="H18" s="3">
+        <v>8.8423352688550949E-2</v>
+      </c>
+      <c r="I18" s="3">
+        <v>0.11566651985049248</v>
+      </c>
+      <c r="J18" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0.3810066126706862</v>
+      </c>
+      <c r="L18" s="3">
+        <v>0.37286116117435042</v>
+      </c>
+      <c r="M18" s="3">
+        <v>0.3810066126706862</v>
+      </c>
+      <c r="N18" s="3"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:I13 J2:M4 J5:J9 L5:L9 J10:M16" xr:uid="{89F920E6-782C-4A76-9D27-5BF3B977A058}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:I13 J2:M4 J5:J9 L5:L9 J10:M18" xr:uid="{89F920E6-782C-4A76-9D27-5BF3B977A058}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -1579,10 +1532,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{063F8C59-CF5A-47F4-9750-D5E7312776B6}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B1" s="5">
@@ -1604,8 +1557,8 @@
         <v>0.18587517738342285</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="5">
@@ -1634,6 +1587,26 @@
       <formula2>1</formula2>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F069A18C-6DD3-4413-99B9-3AD02F70F32F}">
+  <dimension ref="B2:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1648,6 +1621,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B011C3FEFFEFCF44990405A8404263A2" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3dc4baf5bca6f50981051f1202939c23">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79a1cdf2-2d4f-42d7-aee4-ff0e208e0f4a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1497dbabdd8844cfa90d09d2bdc2ce45" ns2:_="">
     <xsd:import namespace="79a1cdf2-2d4f-42d7-aee4-ff0e208e0f4a"/>
@@ -1791,20 +1770,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B49A0F9-2E81-44C2-A3FE-722A90566CC8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B49A0F9-2E81-44C2-A3FE-722A90566CC8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4048B02C-DCD9-4760-9A3E-6C762E5E0491}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4F85AE-6301-4275-977D-807ADA1E6002}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4F85AE-6301-4275-977D-807ADA1E6002}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4048B02C-DCD9-4760-9A3E-6C762E5E0491}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79a1cdf2-2d4f-42d7-aee4-ff0e208e0f4a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>